<commit_message>
Update profit files after running on 2026-09-13
</commit_message>
<xml_diff>
--- a/data/profit_data.xlsx
+++ b/data/profit_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O292"/>
+  <dimension ref="A1:O293"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -14475,6 +14475,55 @@
         <v>88655.28</v>
       </c>
     </row>
+    <row r="293">
+      <c r="A293" t="inlineStr">
+        <is>
+          <t>09/13/2026</t>
+        </is>
+      </c>
+      <c r="B293" t="n">
+        <v>13601.55</v>
+      </c>
+      <c r="C293" t="n">
+        <v>0.3270410193620817</v>
+      </c>
+      <c r="D293" t="n">
+        <v>0.6729589806379183</v>
+      </c>
+      <c r="E293" t="n">
+        <v>-164.07</v>
+      </c>
+      <c r="F293" t="n">
+        <v>-7.6</v>
+      </c>
+      <c r="G293" t="n">
+        <v>-23063.47</v>
+      </c>
+      <c r="H293" t="n">
+        <v>-71.59</v>
+      </c>
+      <c r="I293" t="n">
+        <v>-654.49</v>
+      </c>
+      <c r="J293" t="n">
+        <v>-12.83</v>
+      </c>
+      <c r="K293" t="n">
+        <v>-23718.06</v>
+      </c>
+      <c r="L293" t="n">
+        <v>-63.55</v>
+      </c>
+      <c r="M293" t="n">
+        <v>0.0374</v>
+      </c>
+      <c r="N293" t="n">
+        <v>0.1218</v>
+      </c>
+      <c r="O293" t="n">
+        <v>88485.92999999999</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update profit files after running on 2026-09-14
</commit_message>
<xml_diff>
--- a/data/profit_data.xlsx
+++ b/data/profit_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O293"/>
+  <dimension ref="A1:O294"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -14524,6 +14524,55 @@
         <v>88485.92999999999</v>
       </c>
     </row>
+    <row r="294">
+      <c r="A294" t="inlineStr">
+        <is>
+          <t>09/14/2026</t>
+        </is>
+      </c>
+      <c r="B294" t="n">
+        <v>13583.4</v>
+      </c>
+      <c r="C294" t="n">
+        <v>0.335100758788644</v>
+      </c>
+      <c r="D294" t="n">
+        <v>0.664899241211356</v>
+      </c>
+      <c r="E294" t="n">
+        <v>-190.61</v>
+      </c>
+      <c r="F294" t="n">
+        <v>-8.82</v>
+      </c>
+      <c r="G294" t="n">
+        <v>-23185.16</v>
+      </c>
+      <c r="H294" t="n">
+        <v>-71.97</v>
+      </c>
+      <c r="I294" t="n">
+        <v>-552.04</v>
+      </c>
+      <c r="J294" t="n">
+        <v>-10.82</v>
+      </c>
+      <c r="K294" t="n">
+        <v>-23737.2</v>
+      </c>
+      <c r="L294" t="n">
+        <v>-63.61</v>
+      </c>
+      <c r="M294" t="n">
+        <v>0.0374</v>
+      </c>
+      <c r="N294" t="n">
+        <v>0.1218</v>
+      </c>
+      <c r="O294" t="n">
+        <v>88485.92999999999</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update profit files after running on 2026-09-15
</commit_message>
<xml_diff>
--- a/data/profit_data.xlsx
+++ b/data/profit_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O294"/>
+  <dimension ref="A1:O295"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -14573,6 +14573,55 @@
         <v>88485.92999999999</v>
       </c>
     </row>
+    <row r="295">
+      <c r="A295" t="inlineStr">
+        <is>
+          <t>09/15/2026</t>
+        </is>
+      </c>
+      <c r="B295" t="n">
+        <v>13353.01</v>
+      </c>
+      <c r="C295" t="n">
+        <v>0.3297700552717132</v>
+      </c>
+      <c r="D295" t="n">
+        <v>0.6702299447282868</v>
+      </c>
+      <c r="E295" t="n">
+        <v>-208.49</v>
+      </c>
+      <c r="F295" t="n">
+        <v>-9.65</v>
+      </c>
+      <c r="G295" t="n">
+        <v>-23267.17</v>
+      </c>
+      <c r="H295" t="n">
+        <v>-72.22</v>
+      </c>
+      <c r="I295" t="n">
+        <v>-699.4299999999999</v>
+      </c>
+      <c r="J295" t="n">
+        <v>-13.71</v>
+      </c>
+      <c r="K295" t="n">
+        <v>-23966.6</v>
+      </c>
+      <c r="L295" t="n">
+        <v>-64.22</v>
+      </c>
+      <c r="M295" t="n">
+        <v>0.0374</v>
+      </c>
+      <c r="N295" t="n">
+        <v>0.1218</v>
+      </c>
+      <c r="O295" t="n">
+        <v>88485.92999999999</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update profit files after running on 2026-09-16
</commit_message>
<xml_diff>
--- a/data/profit_data.xlsx
+++ b/data/profit_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O295"/>
+  <dimension ref="A1:O296"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -14622,6 +14622,55 @@
         <v>88485.92999999999</v>
       </c>
     </row>
+    <row r="296">
+      <c r="A296" t="inlineStr">
+        <is>
+          <t>09/16/2026</t>
+        </is>
+      </c>
+      <c r="B296" t="n">
+        <v>12795.77</v>
+      </c>
+      <c r="C296" t="n">
+        <v>0.3415179889133892</v>
+      </c>
+      <c r="D296" t="n">
+        <v>0.6584820110866108</v>
+      </c>
+      <c r="E296" t="n">
+        <v>-322.71</v>
+      </c>
+      <c r="F296" t="n">
+        <v>-14.94</v>
+      </c>
+      <c r="G296" t="n">
+        <v>-23790.97</v>
+      </c>
+      <c r="H296" t="n">
+        <v>-73.84999999999999</v>
+      </c>
+      <c r="I296" t="n">
+        <v>-732.86</v>
+      </c>
+      <c r="J296" t="n">
+        <v>-14.36</v>
+      </c>
+      <c r="K296" t="n">
+        <v>-24523.83</v>
+      </c>
+      <c r="L296" t="n">
+        <v>-65.70999999999999</v>
+      </c>
+      <c r="M296" t="n">
+        <v>0.0374</v>
+      </c>
+      <c r="N296" t="n">
+        <v>0.1218</v>
+      </c>
+      <c r="O296" t="n">
+        <v>88485.92999999999</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update profit files after running on 2026-09-17
</commit_message>
<xml_diff>
--- a/data/profit_data.xlsx
+++ b/data/profit_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O296"/>
+  <dimension ref="A1:O297"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -14671,6 +14671,55 @@
         <v>88485.92999999999</v>
       </c>
     </row>
+    <row r="297">
+      <c r="A297" t="inlineStr">
+        <is>
+          <t>09/17/2026</t>
+        </is>
+      </c>
+      <c r="B297" t="n">
+        <v>13336.72</v>
+      </c>
+      <c r="C297" t="n">
+        <v>0.3313317007324332</v>
+      </c>
+      <c r="D297" t="n">
+        <v>0.6686682992675668</v>
+      </c>
+      <c r="E297" t="n">
+        <v>-215.41</v>
+      </c>
+      <c r="F297" t="n">
+        <v>-9.970000000000001</v>
+      </c>
+      <c r="G297" t="n">
+        <v>-23298.92</v>
+      </c>
+      <c r="H297" t="n">
+        <v>-72.31999999999999</v>
+      </c>
+      <c r="I297" t="n">
+        <v>-683.97</v>
+      </c>
+      <c r="J297" t="n">
+        <v>-13.4</v>
+      </c>
+      <c r="K297" t="n">
+        <v>-23982.89</v>
+      </c>
+      <c r="L297" t="n">
+        <v>-64.26000000000001</v>
+      </c>
+      <c r="M297" t="n">
+        <v>0.0374</v>
+      </c>
+      <c r="N297" t="n">
+        <v>0.1218</v>
+      </c>
+      <c r="O297" t="n">
+        <v>88485.92999999999</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update profit files after running on 2026-09-18
</commit_message>
<xml_diff>
--- a/data/profit_data.xlsx
+++ b/data/profit_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O297"/>
+  <dimension ref="A1:O298"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -14720,6 +14720,55 @@
         <v>88485.92999999999</v>
       </c>
     </row>
+    <row r="298">
+      <c r="A298" t="inlineStr">
+        <is>
+          <t>09/18/2026</t>
+        </is>
+      </c>
+      <c r="B298" t="n">
+        <v>14292.37</v>
+      </c>
+      <c r="C298" t="n">
+        <v>0.3255063051226627</v>
+      </c>
+      <c r="D298" t="n">
+        <v>0.6744936948773373</v>
+      </c>
+      <c r="E298" t="n">
+        <v>-62.18</v>
+      </c>
+      <c r="F298" t="n">
+        <v>-2.85</v>
+      </c>
+      <c r="G298" t="n">
+        <v>-22601.65</v>
+      </c>
+      <c r="H298" t="n">
+        <v>-70.09999999999999</v>
+      </c>
+      <c r="I298" t="n">
+        <v>-450.59</v>
+      </c>
+      <c r="J298" t="n">
+        <v>-8.83</v>
+      </c>
+      <c r="K298" t="n">
+        <v>-23052.24</v>
+      </c>
+      <c r="L298" t="n">
+        <v>-61.73</v>
+      </c>
+      <c r="M298" t="n">
+        <v>0.0374</v>
+      </c>
+      <c r="N298" t="n">
+        <v>0.1215</v>
+      </c>
+      <c r="O298" t="n">
+        <v>88485.92999999999</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update profit files after running on 2026-09-19
</commit_message>
<xml_diff>
--- a/data/profit_data.xlsx
+++ b/data/profit_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O298"/>
+  <dimension ref="A1:O299"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -14769,6 +14769,55 @@
         <v>88485.92999999999</v>
       </c>
     </row>
+    <row r="299">
+      <c r="A299" t="inlineStr">
+        <is>
+          <t>09/19/2026</t>
+        </is>
+      </c>
+      <c r="B299" t="n">
+        <v>15275.32</v>
+      </c>
+      <c r="C299" t="n">
+        <v>0.3081274800084673</v>
+      </c>
+      <c r="D299" t="n">
+        <v>0.6918725199915327</v>
+      </c>
+      <c r="E299" t="n">
+        <v>142.27</v>
+      </c>
+      <c r="F299" t="n">
+        <v>6.51</v>
+      </c>
+      <c r="G299" t="n">
+        <v>-21673.18</v>
+      </c>
+      <c r="H299" t="n">
+        <v>-67.22</v>
+      </c>
+      <c r="I299" t="n">
+        <v>-396.1</v>
+      </c>
+      <c r="J299" t="n">
+        <v>-7.76</v>
+      </c>
+      <c r="K299" t="n">
+        <v>-22069.28</v>
+      </c>
+      <c r="L299" t="n">
+        <v>-59.1</v>
+      </c>
+      <c r="M299" t="n">
+        <v>0.0374</v>
+      </c>
+      <c r="N299" t="n">
+        <v>0.1215</v>
+      </c>
+      <c r="O299" t="n">
+        <v>88485.92999999999</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update profit files after running on 2026-09-20
</commit_message>
<xml_diff>
--- a/data/profit_data.xlsx
+++ b/data/profit_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O299"/>
+  <dimension ref="A1:O300"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -14818,6 +14818,55 @@
         <v>88485.92999999999</v>
       </c>
     </row>
+    <row r="300">
+      <c r="A300" t="inlineStr">
+        <is>
+          <t>09/20/2026</t>
+        </is>
+      </c>
+      <c r="B300" t="n">
+        <v>15058.1</v>
+      </c>
+      <c r="C300" t="n">
+        <v>0.3145305405468828</v>
+      </c>
+      <c r="D300" t="n">
+        <v>0.6854694594531172</v>
+      </c>
+      <c r="E300" t="n">
+        <v>87.95</v>
+      </c>
+      <c r="F300" t="n">
+        <v>4.03</v>
+      </c>
+      <c r="G300" t="n">
+        <v>-21919.89</v>
+      </c>
+      <c r="H300" t="n">
+        <v>-67.98999999999999</v>
+      </c>
+      <c r="I300" t="n">
+        <v>-441.62</v>
+      </c>
+      <c r="J300" t="n">
+        <v>-8.529999999999999</v>
+      </c>
+      <c r="K300" t="n">
+        <v>-22361.51</v>
+      </c>
+      <c r="L300" t="n">
+        <v>-59.76</v>
+      </c>
+      <c r="M300" t="n">
+        <v>0.0374</v>
+      </c>
+      <c r="N300" t="n">
+        <v>0.1215</v>
+      </c>
+      <c r="O300" t="n">
+        <v>88379.56</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update profit files after running on 2026-09-21
</commit_message>
<xml_diff>
--- a/data/profit_data.xlsx
+++ b/data/profit_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O300"/>
+  <dimension ref="A1:O301"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -14867,6 +14867,55 @@
         <v>88379.56</v>
       </c>
     </row>
+    <row r="301">
+      <c r="A301" t="inlineStr">
+        <is>
+          <t>09/21/2026</t>
+        </is>
+      </c>
+      <c r="B301" t="n">
+        <v>16357.17</v>
+      </c>
+      <c r="C301" t="n">
+        <v>0.307666807334371</v>
+      </c>
+      <c r="D301" t="n">
+        <v>0.692333192665629</v>
+      </c>
+      <c r="E301" t="n">
+        <v>308.76</v>
+      </c>
+      <c r="F301" t="n">
+        <v>14.13</v>
+      </c>
+      <c r="G301" t="n">
+        <v>-20917.15</v>
+      </c>
+      <c r="H301" t="n">
+        <v>-64.88</v>
+      </c>
+      <c r="I301" t="n">
+        <v>-145.29</v>
+      </c>
+      <c r="J301" t="n">
+        <v>-2.81</v>
+      </c>
+      <c r="K301" t="n">
+        <v>-21062.44</v>
+      </c>
+      <c r="L301" t="n">
+        <v>-56.29</v>
+      </c>
+      <c r="M301" t="n">
+        <v>0.0374</v>
+      </c>
+      <c r="N301" t="n">
+        <v>0.1215</v>
+      </c>
+      <c r="O301" t="n">
+        <v>88379.56</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update profit files after running on 2026-09-22
</commit_message>
<xml_diff>
--- a/data/profit_data.xlsx
+++ b/data/profit_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O301"/>
+  <dimension ref="A1:O302"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -14916,6 +14916,55 @@
         <v>88379.56</v>
       </c>
     </row>
+    <row r="302">
+      <c r="A302" t="inlineStr">
+        <is>
+          <t>09/22/2026</t>
+        </is>
+      </c>
+      <c r="B302" t="n">
+        <v>16049.91</v>
+      </c>
+      <c r="C302" t="n">
+        <v>0.3144117313405849</v>
+      </c>
+      <c r="D302" t="n">
+        <v>0.6855882686594151</v>
+      </c>
+      <c r="E302" t="n">
+        <v>238.07</v>
+      </c>
+      <c r="F302" t="n">
+        <v>10.9</v>
+      </c>
+      <c r="G302" t="n">
+        <v>-21238.13</v>
+      </c>
+      <c r="H302" t="n">
+        <v>-65.87</v>
+      </c>
+      <c r="I302" t="n">
+        <v>-131.57</v>
+      </c>
+      <c r="J302" t="n">
+        <v>-2.54</v>
+      </c>
+      <c r="K302" t="n">
+        <v>-21369.7</v>
+      </c>
+      <c r="L302" t="n">
+        <v>-57.11</v>
+      </c>
+      <c r="M302" t="n">
+        <v>0.0374</v>
+      </c>
+      <c r="N302" t="n">
+        <v>0.1215</v>
+      </c>
+      <c r="O302" t="n">
+        <v>88379.56</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update profit files after running on 2026-09-23
</commit_message>
<xml_diff>
--- a/data/profit_data.xlsx
+++ b/data/profit_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O302"/>
+  <dimension ref="A1:O303"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -14965,6 +14965,55 @@
         <v>88379.56</v>
       </c>
     </row>
+    <row r="303">
+      <c r="A303" t="inlineStr">
+        <is>
+          <t>09/23/2026</t>
+        </is>
+      </c>
+      <c r="B303" t="n">
+        <v>15173.22</v>
+      </c>
+      <c r="C303" t="n">
+        <v>0.3249760788236111</v>
+      </c>
+      <c r="D303" t="n">
+        <v>0.6750239211763889</v>
+      </c>
+      <c r="E303" t="n">
+        <v>70.42</v>
+      </c>
+      <c r="F303" t="n">
+        <v>3.22</v>
+      </c>
+      <c r="G303" t="n">
+        <v>-21999.47</v>
+      </c>
+      <c r="H303" t="n">
+        <v>-68.23</v>
+      </c>
+      <c r="I303" t="n">
+        <v>-246.92</v>
+      </c>
+      <c r="J303" t="n">
+        <v>-4.77</v>
+      </c>
+      <c r="K303" t="n">
+        <v>-22246.39</v>
+      </c>
+      <c r="L303" t="n">
+        <v>-59.45</v>
+      </c>
+      <c r="M303" t="n">
+        <v>0.0374</v>
+      </c>
+      <c r="N303" t="n">
+        <v>0.1215</v>
+      </c>
+      <c r="O303" t="n">
+        <v>88379.56</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update profit files after running on 2026-09-24
</commit_message>
<xml_diff>
--- a/data/profit_data.xlsx
+++ b/data/profit_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O303"/>
+  <dimension ref="A1:O304"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -15014,6 +15014,55 @@
         <v>88379.56</v>
       </c>
     </row>
+    <row r="304">
+      <c r="A304" t="inlineStr">
+        <is>
+          <t>09/24/2026</t>
+        </is>
+      </c>
+      <c r="B304" t="n">
+        <v>15689.27</v>
+      </c>
+      <c r="C304" t="n">
+        <v>0.3158987557167292</v>
+      </c>
+      <c r="D304" t="n">
+        <v>0.6841012442832708</v>
+      </c>
+      <c r="E304" t="n">
+        <v>178.49</v>
+      </c>
+      <c r="F304" t="n">
+        <v>8.17</v>
+      </c>
+      <c r="G304" t="n">
+        <v>-21508.71</v>
+      </c>
+      <c r="H304" t="n">
+        <v>-66.70999999999999</v>
+      </c>
+      <c r="I304" t="n">
+        <v>-220.95</v>
+      </c>
+      <c r="J304" t="n">
+        <v>-4.27</v>
+      </c>
+      <c r="K304" t="n">
+        <v>-21729.66</v>
+      </c>
+      <c r="L304" t="n">
+        <v>-58.07</v>
+      </c>
+      <c r="M304" t="n">
+        <v>0.0374</v>
+      </c>
+      <c r="N304" t="n">
+        <v>0.1215</v>
+      </c>
+      <c r="O304" t="n">
+        <v>88379.56</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update profit files after running on 2026-09-25
</commit_message>
<xml_diff>
--- a/data/profit_data.xlsx
+++ b/data/profit_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O304"/>
+  <dimension ref="A1:O305"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -15063,6 +15063,55 @@
         <v>88379.56</v>
       </c>
     </row>
+    <row r="305">
+      <c r="A305" t="inlineStr">
+        <is>
+          <t>09/25/2026</t>
+        </is>
+      </c>
+      <c r="B305" t="n">
+        <v>15931.42</v>
+      </c>
+      <c r="C305" t="n">
+        <v>0.3078790842800952</v>
+      </c>
+      <c r="D305" t="n">
+        <v>0.6921209157199048</v>
+      </c>
+      <c r="E305" t="n">
+        <v>237.98</v>
+      </c>
+      <c r="F305" t="n">
+        <v>10.77</v>
+      </c>
+      <c r="G305" t="n">
+        <v>-21240.29</v>
+      </c>
+      <c r="H305" t="n">
+        <v>-65.83</v>
+      </c>
+      <c r="I305" t="n">
+        <v>-272.9</v>
+      </c>
+      <c r="J305" t="n">
+        <v>-5.27</v>
+      </c>
+      <c r="K305" t="n">
+        <v>-21513.19</v>
+      </c>
+      <c r="L305" t="n">
+        <v>-57.45</v>
+      </c>
+      <c r="M305" t="n">
+        <v>0.0374</v>
+      </c>
+      <c r="N305" t="n">
+        <v>0.1214</v>
+      </c>
+      <c r="O305" t="n">
+        <v>88379.56</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update profit files after running on 2026-09-26
</commit_message>
<xml_diff>
--- a/data/profit_data.xlsx
+++ b/data/profit_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O305"/>
+  <dimension ref="A1:O306"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -15112,6 +15112,55 @@
         <v>88379.56</v>
       </c>
     </row>
+    <row r="306">
+      <c r="A306" t="inlineStr">
+        <is>
+          <t>09/26/2026</t>
+        </is>
+      </c>
+      <c r="B306" t="n">
+        <v>17652.49</v>
+      </c>
+      <c r="C306" t="n">
+        <v>0.279260550941083</v>
+      </c>
+      <c r="D306" t="n">
+        <v>0.720739449058917</v>
+      </c>
+      <c r="E306" t="n">
+        <v>614.6</v>
+      </c>
+      <c r="F306" t="n">
+        <v>27.81</v>
+      </c>
+      <c r="G306" t="n">
+        <v>-19543.91</v>
+      </c>
+      <c r="H306" t="n">
+        <v>-60.57</v>
+      </c>
+      <c r="I306" t="n">
+        <v>-248.21</v>
+      </c>
+      <c r="J306" t="n">
+        <v>-4.79</v>
+      </c>
+      <c r="K306" t="n">
+        <v>-19792.12</v>
+      </c>
+      <c r="L306" t="n">
+        <v>-52.86</v>
+      </c>
+      <c r="M306" t="n">
+        <v>0.0374</v>
+      </c>
+      <c r="N306" t="n">
+        <v>0.1214</v>
+      </c>
+      <c r="O306" t="n">
+        <v>88379.56</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update profit files after running on 2026-09-27
</commit_message>
<xml_diff>
--- a/data/profit_data.xlsx
+++ b/data/profit_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O306"/>
+  <dimension ref="A1:O307"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -15161,6 +15161,55 @@
         <v>88379.56</v>
       </c>
     </row>
+    <row r="307">
+      <c r="A307" t="inlineStr">
+        <is>
+          <t>09/27/2026</t>
+        </is>
+      </c>
+      <c r="B307" t="n">
+        <v>17649.92</v>
+      </c>
+      <c r="C307" t="n">
+        <v>0.2845786028228841</v>
+      </c>
+      <c r="D307" t="n">
+        <v>0.7154213971771159</v>
+      </c>
+      <c r="E307" t="n">
+        <v>593.35</v>
+      </c>
+      <c r="F307" t="n">
+        <v>26.85</v>
+      </c>
+      <c r="G307" t="n">
+        <v>-19639.63</v>
+      </c>
+      <c r="H307" t="n">
+        <v>-60.87</v>
+      </c>
+      <c r="I307" t="n">
+        <v>-230.06</v>
+      </c>
+      <c r="J307" t="n">
+        <v>-4.38</v>
+      </c>
+      <c r="K307" t="n">
+        <v>-19869.69</v>
+      </c>
+      <c r="L307" t="n">
+        <v>-52.96</v>
+      </c>
+      <c r="M307" t="n">
+        <v>0.0374</v>
+      </c>
+      <c r="N307" t="n">
+        <v>0.1214</v>
+      </c>
+      <c r="O307" t="n">
+        <v>88342.17</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update profit files after running on 2026-09-28
</commit_message>
<xml_diff>
--- a/data/profit_data.xlsx
+++ b/data/profit_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O307"/>
+  <dimension ref="A1:O308"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -15210,6 +15210,55 @@
         <v>88342.17</v>
       </c>
     </row>
+    <row r="308">
+      <c r="A308" t="inlineStr">
+        <is>
+          <t>09/28/2026</t>
+        </is>
+      </c>
+      <c r="B308" t="n">
+        <v>16901.21</v>
+      </c>
+      <c r="C308" t="n">
+        <v>0.2942615355716088</v>
+      </c>
+      <c r="D308" t="n">
+        <v>0.7057384644283912</v>
+      </c>
+      <c r="E308" t="n">
+        <v>438.1</v>
+      </c>
+      <c r="F308" t="n">
+        <v>19.82</v>
+      </c>
+      <c r="G308" t="n">
+        <v>-20338.92</v>
+      </c>
+      <c r="H308" t="n">
+        <v>-63.03</v>
+      </c>
+      <c r="I308" t="n">
+        <v>-279.47</v>
+      </c>
+      <c r="J308" t="n">
+        <v>-5.32</v>
+      </c>
+      <c r="K308" t="n">
+        <v>-20618.39</v>
+      </c>
+      <c r="L308" t="n">
+        <v>-54.95</v>
+      </c>
+      <c r="M308" t="n">
+        <v>0.0374</v>
+      </c>
+      <c r="N308" t="n">
+        <v>0.1214</v>
+      </c>
+      <c r="O308" t="n">
+        <v>88342.17</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update profit files after running on 2026-09-29
</commit_message>
<xml_diff>
--- a/data/profit_data.xlsx
+++ b/data/profit_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O308"/>
+  <dimension ref="A1:O309"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -15259,6 +15259,55 @@
         <v>88342.17</v>
       </c>
     </row>
+    <row r="309">
+      <c r="A309" t="inlineStr">
+        <is>
+          <t>09/29/2026</t>
+        </is>
+      </c>
+      <c r="B309" t="n">
+        <v>16644.24</v>
+      </c>
+      <c r="C309" t="n">
+        <v>0.2966247662814455</v>
+      </c>
+      <c r="D309" t="n">
+        <v>0.7033752337185545</v>
+      </c>
+      <c r="E309" t="n">
+        <v>389.1</v>
+      </c>
+      <c r="F309" t="n">
+        <v>17.61</v>
+      </c>
+      <c r="G309" t="n">
+        <v>-20559.61</v>
+      </c>
+      <c r="H309" t="n">
+        <v>-63.72</v>
+      </c>
+      <c r="I309" t="n">
+        <v>-315.82</v>
+      </c>
+      <c r="J309" t="n">
+        <v>-6.01</v>
+      </c>
+      <c r="K309" t="n">
+        <v>-20875.37</v>
+      </c>
+      <c r="L309" t="n">
+        <v>-55.64</v>
+      </c>
+      <c r="M309" t="n">
+        <v>0.0374</v>
+      </c>
+      <c r="N309" t="n">
+        <v>0.1214</v>
+      </c>
+      <c r="O309" t="n">
+        <v>88342.17</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update profit files after running on 2026-09-30
</commit_message>
<xml_diff>
--- a/data/profit_data.xlsx
+++ b/data/profit_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O309"/>
+  <dimension ref="A1:O310"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -15308,6 +15308,55 @@
         <v>88342.17</v>
       </c>
     </row>
+    <row r="310">
+      <c r="A310" t="inlineStr">
+        <is>
+          <t>09/30/2026</t>
+        </is>
+      </c>
+      <c r="B310" t="n">
+        <v>16421.32</v>
+      </c>
+      <c r="C310" t="n">
+        <v>0.3040776351389318</v>
+      </c>
+      <c r="D310" t="n">
+        <v>0.6959223648610682</v>
+      </c>
+      <c r="E310" t="n">
+        <v>327.12</v>
+      </c>
+      <c r="F310" t="n">
+        <v>14.8</v>
+      </c>
+      <c r="G310" t="n">
+        <v>-20838.8</v>
+      </c>
+      <c r="H310" t="n">
+        <v>-64.58</v>
+      </c>
+      <c r="I310" t="n">
+        <v>-259.49</v>
+      </c>
+      <c r="J310" t="n">
+        <v>-4.94</v>
+      </c>
+      <c r="K310" t="n">
+        <v>-21098.29</v>
+      </c>
+      <c r="L310" t="n">
+        <v>-56.23</v>
+      </c>
+      <c r="M310" t="n">
+        <v>0.0374</v>
+      </c>
+      <c r="N310" t="n">
+        <v>0.1214</v>
+      </c>
+      <c r="O310" t="n">
+        <v>88342.17</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update profit files after running on 2026-10-01
</commit_message>
<xml_diff>
--- a/data/profit_data.xlsx
+++ b/data/profit_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O310"/>
+  <dimension ref="A1:O311"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -15357,6 +15357,55 @@
         <v>88342.17</v>
       </c>
     </row>
+    <row r="311">
+      <c r="A311" t="inlineStr">
+        <is>
+          <t>10/01/2026</t>
+        </is>
+      </c>
+      <c r="B311" t="n">
+        <v>16087.64</v>
+      </c>
+      <c r="C311" t="n">
+        <v>0.3137735240541877</v>
+      </c>
+      <c r="D311" t="n">
+        <v>0.6862264759458123</v>
+      </c>
+      <c r="E311" t="n">
+        <v>240.94</v>
+      </c>
+      <c r="F311" t="n">
+        <v>10.9</v>
+      </c>
+      <c r="G311" t="n">
+        <v>-21227</v>
+      </c>
+      <c r="H311" t="n">
+        <v>-65.79000000000001</v>
+      </c>
+      <c r="I311" t="n">
+        <v>-204.98</v>
+      </c>
+      <c r="J311" t="n">
+        <v>-3.9</v>
+      </c>
+      <c r="K311" t="n">
+        <v>-21431.98</v>
+      </c>
+      <c r="L311" t="n">
+        <v>-57.12</v>
+      </c>
+      <c r="M311" t="n">
+        <v>0.0374</v>
+      </c>
+      <c r="N311" t="n">
+        <v>0.1214</v>
+      </c>
+      <c r="O311" t="n">
+        <v>88342.17</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update profit files after running on 2026-10-02
</commit_message>
<xml_diff>
--- a/data/profit_data.xlsx
+++ b/data/profit_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O311"/>
+  <dimension ref="A1:O312"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -15406,6 +15406,55 @@
         <v>88342.17</v>
       </c>
     </row>
+    <row r="312">
+      <c r="A312" t="inlineStr">
+        <is>
+          <t>10/02/2026</t>
+        </is>
+      </c>
+      <c r="B312" t="n">
+        <v>16397.1</v>
+      </c>
+      <c r="C312" t="n">
+        <v>0.3071082685559827</v>
+      </c>
+      <c r="D312" t="n">
+        <v>0.6928917314440173</v>
+      </c>
+      <c r="E312" t="n">
+        <v>301.59</v>
+      </c>
+      <c r="F312" t="n">
+        <v>13.34</v>
+      </c>
+      <c r="G312" t="n">
+        <v>-20955.34</v>
+      </c>
+      <c r="H312" t="n">
+        <v>-64.84</v>
+      </c>
+      <c r="I312" t="n">
+        <v>-217.16</v>
+      </c>
+      <c r="J312" t="n">
+        <v>-4.13</v>
+      </c>
+      <c r="K312" t="n">
+        <v>-21172.5</v>
+      </c>
+      <c r="L312" t="n">
+        <v>-56.36</v>
+      </c>
+      <c r="M312" t="n">
+        <v>0.0375</v>
+      </c>
+      <c r="N312" t="n">
+        <v>0.121</v>
+      </c>
+      <c r="O312" t="n">
+        <v>88342.17</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update profit files after running on 2026-10-03
</commit_message>
<xml_diff>
--- a/data/profit_data.xlsx
+++ b/data/profit_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O312"/>
+  <dimension ref="A1:O313"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -15455,6 +15455,55 @@
         <v>88342.17</v>
       </c>
     </row>
+    <row r="313">
+      <c r="A313" t="inlineStr">
+        <is>
+          <t>10/03/2026</t>
+        </is>
+      </c>
+      <c r="B313" t="n">
+        <v>16381.97</v>
+      </c>
+      <c r="C313" t="n">
+        <v>0.3079356173834555</v>
+      </c>
+      <c r="D313" t="n">
+        <v>0.6920643826165445</v>
+      </c>
+      <c r="E313" t="n">
+        <v>296.17</v>
+      </c>
+      <c r="F313" t="n">
+        <v>13.1</v>
+      </c>
+      <c r="G313" t="n">
+        <v>-20979.38</v>
+      </c>
+      <c r="H313" t="n">
+        <v>-64.92</v>
+      </c>
+      <c r="I313" t="n">
+        <v>-208.26</v>
+      </c>
+      <c r="J313" t="n">
+        <v>-3.96</v>
+      </c>
+      <c r="K313" t="n">
+        <v>-21187.64</v>
+      </c>
+      <c r="L313" t="n">
+        <v>-56.4</v>
+      </c>
+      <c r="M313" t="n">
+        <v>0.0375</v>
+      </c>
+      <c r="N313" t="n">
+        <v>0.121</v>
+      </c>
+      <c r="O313" t="n">
+        <v>88342.17</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update profit files after running on 2026-10-04
</commit_message>
<xml_diff>
--- a/data/profit_data.xlsx
+++ b/data/profit_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O313"/>
+  <dimension ref="A1:O314"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -15504,6 +15504,55 @@
         <v>88342.17</v>
       </c>
     </row>
+    <row r="314">
+      <c r="A314" t="inlineStr">
+        <is>
+          <t>10/04/2026</t>
+        </is>
+      </c>
+      <c r="B314" t="n">
+        <v>16397.41</v>
+      </c>
+      <c r="C314" t="n">
+        <v>0.3123335851411533</v>
+      </c>
+      <c r="D314" t="n">
+        <v>0.6876664148588467</v>
+      </c>
+      <c r="E314" t="n">
+        <v>282.32</v>
+      </c>
+      <c r="F314" t="n">
+        <v>12.49</v>
+      </c>
+      <c r="G314" t="n">
+        <v>-21040.81</v>
+      </c>
+      <c r="H314" t="n">
+        <v>-65.11</v>
+      </c>
+      <c r="I314" t="n">
+        <v>-181.39</v>
+      </c>
+      <c r="J314" t="n">
+        <v>-3.42</v>
+      </c>
+      <c r="K314" t="n">
+        <v>-21222.2</v>
+      </c>
+      <c r="L314" t="n">
+        <v>-56.41</v>
+      </c>
+      <c r="M314" t="n">
+        <v>0.0375</v>
+      </c>
+      <c r="N314" t="n">
+        <v>0.121</v>
+      </c>
+      <c r="O314" t="n">
+        <v>88321.07000000001</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update profit files after running on 2026-10-05
</commit_message>
<xml_diff>
--- a/data/profit_data.xlsx
+++ b/data/profit_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O314"/>
+  <dimension ref="A1:O315"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -15553,6 +15553,55 @@
         <v>88321.07000000001</v>
       </c>
     </row>
+    <row r="315">
+      <c r="A315" t="inlineStr">
+        <is>
+          <t>10/05/2026</t>
+        </is>
+      </c>
+      <c r="B315" t="n">
+        <v>16762.32</v>
+      </c>
+      <c r="C315" t="n">
+        <v>0.3072278307758125</v>
+      </c>
+      <c r="D315" t="n">
+        <v>0.6927721692241875</v>
+      </c>
+      <c r="E315" t="n">
+        <v>358.19</v>
+      </c>
+      <c r="F315" t="n">
+        <v>15.85</v>
+      </c>
+      <c r="G315" t="n">
+        <v>-20704.29</v>
+      </c>
+      <c r="H315" t="n">
+        <v>-64.06999999999999</v>
+      </c>
+      <c r="I315" t="n">
+        <v>-153</v>
+      </c>
+      <c r="J315" t="n">
+        <v>-2.89</v>
+      </c>
+      <c r="K315" t="n">
+        <v>-20857.29</v>
+      </c>
+      <c r="L315" t="n">
+        <v>-55.44</v>
+      </c>
+      <c r="M315" t="n">
+        <v>0.0375</v>
+      </c>
+      <c r="N315" t="n">
+        <v>0.121</v>
+      </c>
+      <c r="O315" t="n">
+        <v>88321.07000000001</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update profit files after running on 2026-10-06
</commit_message>
<xml_diff>
--- a/data/profit_data.xlsx
+++ b/data/profit_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O315"/>
+  <dimension ref="A1:O316"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -15602,6 +15602,55 @@
         <v>88321.07000000001</v>
       </c>
     </row>
+    <row r="316">
+      <c r="A316" t="inlineStr">
+        <is>
+          <t>10/06/2026</t>
+        </is>
+      </c>
+      <c r="B316" t="n">
+        <v>16754.46</v>
+      </c>
+      <c r="C316" t="n">
+        <v>0.307380959125505</v>
+      </c>
+      <c r="D316" t="n">
+        <v>0.692619040874495</v>
+      </c>
+      <c r="E316" t="n">
+        <v>356.39</v>
+      </c>
+      <c r="F316" t="n">
+        <v>15.77</v>
+      </c>
+      <c r="G316" t="n">
+        <v>-20712.3</v>
+      </c>
+      <c r="H316" t="n">
+        <v>-64.09</v>
+      </c>
+      <c r="I316" t="n">
+        <v>-152.86</v>
+      </c>
+      <c r="J316" t="n">
+        <v>-2.88</v>
+      </c>
+      <c r="K316" t="n">
+        <v>-20865.15</v>
+      </c>
+      <c r="L316" t="n">
+        <v>-55.46</v>
+      </c>
+      <c r="M316" t="n">
+        <v>0.0375</v>
+      </c>
+      <c r="N316" t="n">
+        <v>0.121</v>
+      </c>
+      <c r="O316" t="n">
+        <v>88321.07000000001</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update profit files after running on 2026-10-07
</commit_message>
<xml_diff>
--- a/data/profit_data.xlsx
+++ b/data/profit_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O316"/>
+  <dimension ref="A1:O317"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -15651,6 +15651,55 @@
         <v>88321.07000000001</v>
       </c>
     </row>
+    <row r="317">
+      <c r="A317" t="inlineStr">
+        <is>
+          <t>10/07/2026</t>
+        </is>
+      </c>
+      <c r="B317" t="n">
+        <v>15675.7</v>
+      </c>
+      <c r="C317" t="n">
+        <v>0.3190076559743615</v>
+      </c>
+      <c r="D317" t="n">
+        <v>0.6809923440256385</v>
+      </c>
+      <c r="E317" t="n">
+        <v>146.84</v>
+      </c>
+      <c r="F317" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="G317" t="n">
+        <v>-21641.73</v>
+      </c>
+      <c r="H317" t="n">
+        <v>-66.97</v>
+      </c>
+      <c r="I317" t="n">
+        <v>-302.18</v>
+      </c>
+      <c r="J317" t="n">
+        <v>-5.7</v>
+      </c>
+      <c r="K317" t="n">
+        <v>-21943.91</v>
+      </c>
+      <c r="L317" t="n">
+        <v>-58.33</v>
+      </c>
+      <c r="M317" t="n">
+        <v>0.0375</v>
+      </c>
+      <c r="N317" t="n">
+        <v>0.121</v>
+      </c>
+      <c r="O317" t="n">
+        <v>88321.07000000001</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update profit files after running on 2026-10-08
</commit_message>
<xml_diff>
--- a/data/profit_data.xlsx
+++ b/data/profit_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O317"/>
+  <dimension ref="A1:O318"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -15700,6 +15700,55 @@
         <v>88321.07000000001</v>
       </c>
     </row>
+    <row r="318">
+      <c r="A318" t="inlineStr">
+        <is>
+          <t>10/08/2026</t>
+        </is>
+      </c>
+      <c r="B318" t="n">
+        <v>15211.09</v>
+      </c>
+      <c r="C318" t="n">
+        <v>0.3208748362056056</v>
+      </c>
+      <c r="D318" t="n">
+        <v>0.6791251637943944</v>
+      </c>
+      <c r="E318" t="n">
+        <v>69.16</v>
+      </c>
+      <c r="F318" t="n">
+        <v>3.06</v>
+      </c>
+      <c r="G318" t="n">
+        <v>-21986.26</v>
+      </c>
+      <c r="H318" t="n">
+        <v>-68.03</v>
+      </c>
+      <c r="I318" t="n">
+        <v>-421.87</v>
+      </c>
+      <c r="J318" t="n">
+        <v>-7.96</v>
+      </c>
+      <c r="K318" t="n">
+        <v>-22408.13</v>
+      </c>
+      <c r="L318" t="n">
+        <v>-59.57</v>
+      </c>
+      <c r="M318" t="n">
+        <v>0.0375</v>
+      </c>
+      <c r="N318" t="n">
+        <v>0.121</v>
+      </c>
+      <c r="O318" t="n">
+        <v>88321.07000000001</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update profit files after running on 2026-10-09
</commit_message>
<xml_diff>
--- a/data/profit_data.xlsx
+++ b/data/profit_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O318"/>
+  <dimension ref="A1:O319"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -15749,6 +15749,55 @@
         <v>88321.07000000001</v>
       </c>
     </row>
+    <row r="319">
+      <c r="A319" t="inlineStr">
+        <is>
+          <t>10/09/2026</t>
+        </is>
+      </c>
+      <c r="B319" t="n">
+        <v>16108</v>
+      </c>
+      <c r="C319" t="n">
+        <v>0.3080389853798325</v>
+      </c>
+      <c r="D319" t="n">
+        <v>0.6919610146201675</v>
+      </c>
+      <c r="E319" t="n">
+        <v>243.15</v>
+      </c>
+      <c r="F319" t="n">
+        <v>10.53</v>
+      </c>
+      <c r="G319" t="n">
+        <v>-21220.65</v>
+      </c>
+      <c r="H319" t="n">
+        <v>-65.56</v>
+      </c>
+      <c r="I319" t="n">
+        <v>-340.95</v>
+      </c>
+      <c r="J319" t="n">
+        <v>-6.43</v>
+      </c>
+      <c r="K319" t="n">
+        <v>-21561.61</v>
+      </c>
+      <c r="L319" t="n">
+        <v>-57.24</v>
+      </c>
+      <c r="M319" t="n">
+        <v>0.0376</v>
+      </c>
+      <c r="N319" t="n">
+        <v>0.1206</v>
+      </c>
+      <c r="O319" t="n">
+        <v>88321.07000000001</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update profit files after running on 2026-10-10
</commit_message>
<xml_diff>
--- a/data/profit_data.xlsx
+++ b/data/profit_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O319"/>
+  <dimension ref="A1:O320"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -15798,6 +15798,55 @@
         <v>88321.07000000001</v>
       </c>
     </row>
+    <row r="320">
+      <c r="A320" t="inlineStr">
+        <is>
+          <t>10/10/2026</t>
+        </is>
+      </c>
+      <c r="B320" t="n">
+        <v>16015.81</v>
+      </c>
+      <c r="C320" t="n">
+        <v>0.3110923708306992</v>
+      </c>
+      <c r="D320" t="n">
+        <v>0.6889076291693008</v>
+      </c>
+      <c r="E320" t="n">
+        <v>217.33</v>
+      </c>
+      <c r="F320" t="n">
+        <v>9.41</v>
+      </c>
+      <c r="G320" t="n">
+        <v>-21333.34</v>
+      </c>
+      <c r="H320" t="n">
+        <v>-65.91</v>
+      </c>
+      <c r="I320" t="n">
+        <v>-320.45</v>
+      </c>
+      <c r="J320" t="n">
+        <v>-6.04</v>
+      </c>
+      <c r="K320" t="n">
+        <v>-21653.79</v>
+      </c>
+      <c r="L320" t="n">
+        <v>-57.48</v>
+      </c>
+      <c r="M320" t="n">
+        <v>0.0376</v>
+      </c>
+      <c r="N320" t="n">
+        <v>0.1206</v>
+      </c>
+      <c r="O320" t="n">
+        <v>88321.07000000001</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update profit files after running on 2026-10-11
</commit_message>
<xml_diff>
--- a/data/profit_data.xlsx
+++ b/data/profit_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O320"/>
+  <dimension ref="A1:O321"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -15847,6 +15847,55 @@
         <v>88321.07000000001</v>
       </c>
     </row>
+    <row r="321">
+      <c r="A321" t="inlineStr">
+        <is>
+          <t>10/11/2026</t>
+        </is>
+      </c>
+      <c r="B321" t="n">
+        <v>16234.17</v>
+      </c>
+      <c r="C321" t="n">
+        <v>0.3134165023339828</v>
+      </c>
+      <c r="D321" t="n">
+        <v>0.6865834976660172</v>
+      </c>
+      <c r="E321" t="n">
+        <v>243.15</v>
+      </c>
+      <c r="F321" t="n">
+        <v>10.53</v>
+      </c>
+      <c r="G321" t="n">
+        <v>-21220.65</v>
+      </c>
+      <c r="H321" t="n">
+        <v>-65.56</v>
+      </c>
+      <c r="I321" t="n">
+        <v>-264.79</v>
+      </c>
+      <c r="J321" t="n">
+        <v>-4.95</v>
+      </c>
+      <c r="K321" t="n">
+        <v>-21485.44</v>
+      </c>
+      <c r="L321" t="n">
+        <v>-56.96</v>
+      </c>
+      <c r="M321" t="n">
+        <v>0.0376</v>
+      </c>
+      <c r="N321" t="n">
+        <v>0.1206</v>
+      </c>
+      <c r="O321" t="n">
+        <v>88281.08</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update profit files after running on 2026-10-12
</commit_message>
<xml_diff>
--- a/data/profit_data.xlsx
+++ b/data/profit_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O321"/>
+  <dimension ref="A1:O322"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -15896,6 +15896,55 @@
         <v>88281.08</v>
       </c>
     </row>
+    <row r="322">
+      <c r="A322" t="inlineStr">
+        <is>
+          <t>10/12/2026</t>
+        </is>
+      </c>
+      <c r="B322" t="n">
+        <v>15548.81</v>
+      </c>
+      <c r="C322" t="n">
+        <v>0.3233619234207854</v>
+      </c>
+      <c r="D322" t="n">
+        <v>0.6766380765792146</v>
+      </c>
+      <c r="E322" t="n">
+        <v>99.94</v>
+      </c>
+      <c r="F322" t="n">
+        <v>4.33</v>
+      </c>
+      <c r="G322" t="n">
+        <v>-21845.84</v>
+      </c>
+      <c r="H322" t="n">
+        <v>-67.48999999999999</v>
+      </c>
+      <c r="I322" t="n">
+        <v>-324.82</v>
+      </c>
+      <c r="J322" t="n">
+        <v>-6.07</v>
+      </c>
+      <c r="K322" t="n">
+        <v>-22170.8</v>
+      </c>
+      <c r="L322" t="n">
+        <v>-58.78</v>
+      </c>
+      <c r="M322" t="n">
+        <v>0.0376</v>
+      </c>
+      <c r="N322" t="n">
+        <v>0.1206</v>
+      </c>
+      <c r="O322" t="n">
+        <v>88281.08</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update profit files after running on 2026-10-13
</commit_message>
<xml_diff>
--- a/data/profit_data.xlsx
+++ b/data/profit_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O322"/>
+  <dimension ref="A1:O323"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -15945,6 +15945,55 @@
         <v>88281.08</v>
       </c>
     </row>
+    <row r="323">
+      <c r="A323" t="inlineStr">
+        <is>
+          <t>10/13/2026</t>
+        </is>
+      </c>
+      <c r="B323" t="n">
+        <v>15300.96</v>
+      </c>
+      <c r="C323" t="n">
+        <v>0.3292360346670573</v>
+      </c>
+      <c r="D323" t="n">
+        <v>0.6707639653329427</v>
+      </c>
+      <c r="E323" t="n">
+        <v>40.94</v>
+      </c>
+      <c r="F323" t="n">
+        <v>1.77</v>
+      </c>
+      <c r="G323" t="n">
+        <v>-22103.43</v>
+      </c>
+      <c r="H323" t="n">
+        <v>-68.29000000000001</v>
+      </c>
+      <c r="I323" t="n">
+        <v>-315.22</v>
+      </c>
+      <c r="J323" t="n">
+        <v>-5.89</v>
+      </c>
+      <c r="K323" t="n">
+        <v>-22418.65</v>
+      </c>
+      <c r="L323" t="n">
+        <v>-59.44</v>
+      </c>
+      <c r="M323" t="n">
+        <v>0.0376</v>
+      </c>
+      <c r="N323" t="n">
+        <v>0.1206</v>
+      </c>
+      <c r="O323" t="n">
+        <v>88281.08</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update profit files after running on 2026-10-14
</commit_message>
<xml_diff>
--- a/data/profit_data.xlsx
+++ b/data/profit_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O323"/>
+  <dimension ref="A1:O324"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -15994,6 +15994,55 @@
         <v>88281.08</v>
       </c>
     </row>
+    <row r="324">
+      <c r="A324" t="inlineStr">
+        <is>
+          <t>10/14/2026</t>
+        </is>
+      </c>
+      <c r="B324" t="n">
+        <v>15052.99</v>
+      </c>
+      <c r="C324" t="n">
+        <v>0.3297730476110831</v>
+      </c>
+      <c r="D324" t="n">
+        <v>0.6702269523889169</v>
+      </c>
+      <c r="E324" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="F324" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="G324" t="n">
+        <v>-22277.84</v>
+      </c>
+      <c r="H324" t="n">
+        <v>-68.83</v>
+      </c>
+      <c r="I324" t="n">
+        <v>-388.78</v>
+      </c>
+      <c r="J324" t="n">
+        <v>-7.26</v>
+      </c>
+      <c r="K324" t="n">
+        <v>-22666.62</v>
+      </c>
+      <c r="L324" t="n">
+        <v>-60.09</v>
+      </c>
+      <c r="M324" t="n">
+        <v>0.0376</v>
+      </c>
+      <c r="N324" t="n">
+        <v>0.1206</v>
+      </c>
+      <c r="O324" t="n">
+        <v>88281.08</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update profit files after running on 2026-10-15
</commit_message>
<xml_diff>
--- a/data/profit_data.xlsx
+++ b/data/profit_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O324"/>
+  <dimension ref="A1:O325"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -16043,6 +16043,55 @@
         <v>88281.08</v>
       </c>
     </row>
+    <row r="325">
+      <c r="A325" t="inlineStr">
+        <is>
+          <t>10/15/2026</t>
+        </is>
+      </c>
+      <c r="B325" t="n">
+        <v>14531.47</v>
+      </c>
+      <c r="C325" t="n">
+        <v>0.3417256356137524</v>
+      </c>
+      <c r="D325" t="n">
+        <v>0.6582743643862476</v>
+      </c>
+      <c r="E325" t="n">
+        <v>-118.87</v>
+      </c>
+      <c r="F325" t="n">
+        <v>-5.15</v>
+      </c>
+      <c r="G325" t="n">
+        <v>-22801.07</v>
+      </c>
+      <c r="H325" t="n">
+        <v>-70.45</v>
+      </c>
+      <c r="I325" t="n">
+        <v>-387.08</v>
+      </c>
+      <c r="J325" t="n">
+        <v>-7.23</v>
+      </c>
+      <c r="K325" t="n">
+        <v>-23188.15</v>
+      </c>
+      <c r="L325" t="n">
+        <v>-61.48</v>
+      </c>
+      <c r="M325" t="n">
+        <v>0.0376</v>
+      </c>
+      <c r="N325" t="n">
+        <v>0.1206</v>
+      </c>
+      <c r="O325" t="n">
+        <v>88281.08</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update profit files after running on 2026-10-16
</commit_message>
<xml_diff>
--- a/data/profit_data.xlsx
+++ b/data/profit_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O325"/>
+  <dimension ref="A1:O326"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -16092,6 +16092,55 @@
         <v>88281.08</v>
       </c>
     </row>
+    <row r="326">
+      <c r="A326" t="inlineStr">
+        <is>
+          <t>10/16/2026</t>
+        </is>
+      </c>
+      <c r="B326" t="n">
+        <v>14906.35</v>
+      </c>
+      <c r="C326" t="n">
+        <v>0.3315036790219348</v>
+      </c>
+      <c r="D326" t="n">
+        <v>0.6684963209780652</v>
+      </c>
+      <c r="E326" t="n">
+        <v>-38.64</v>
+      </c>
+      <c r="F326" t="n">
+        <v>-1.64</v>
+      </c>
+      <c r="G326" t="n">
+        <v>-22451.92</v>
+      </c>
+      <c r="H326" t="n">
+        <v>-69.26000000000001</v>
+      </c>
+      <c r="I326" t="n">
+        <v>-411.34</v>
+      </c>
+      <c r="J326" t="n">
+        <v>-7.68</v>
+      </c>
+      <c r="K326" t="n">
+        <v>-22863.26</v>
+      </c>
+      <c r="L326" t="n">
+        <v>-60.53</v>
+      </c>
+      <c r="M326" t="n">
+        <v>0.0376</v>
+      </c>
+      <c r="N326" t="n">
+        <v>0.1202</v>
+      </c>
+      <c r="O326" t="n">
+        <v>88281.08</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update profit files after running on 2026-10-17
</commit_message>
<xml_diff>
--- a/data/profit_data.xlsx
+++ b/data/profit_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O326"/>
+  <dimension ref="A1:O327"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -16141,6 +16141,55 @@
         <v>88281.08</v>
       </c>
     </row>
+    <row r="327">
+      <c r="A327" t="inlineStr">
+        <is>
+          <t>10/17/2026</t>
+        </is>
+      </c>
+      <c r="B327" t="n">
+        <v>14539.37</v>
+      </c>
+      <c r="C327" t="n">
+        <v>0.3396711780668573</v>
+      </c>
+      <c r="D327" t="n">
+        <v>0.6603288219331427</v>
+      </c>
+      <c r="E327" t="n">
+        <v>-123.45</v>
+      </c>
+      <c r="F327" t="n">
+        <v>-5.23</v>
+      </c>
+      <c r="G327" t="n">
+        <v>-22815.99</v>
+      </c>
+      <c r="H327" t="n">
+        <v>-70.38</v>
+      </c>
+      <c r="I327" t="n">
+        <v>-414.25</v>
+      </c>
+      <c r="J327" t="n">
+        <v>-7.74</v>
+      </c>
+      <c r="K327" t="n">
+        <v>-23230.24</v>
+      </c>
+      <c r="L327" t="n">
+        <v>-61.51</v>
+      </c>
+      <c r="M327" t="n">
+        <v>0.0376</v>
+      </c>
+      <c r="N327" t="n">
+        <v>0.1202</v>
+      </c>
+      <c r="O327" t="n">
+        <v>88281.08</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update profit files after running on 2026-10-18
</commit_message>
<xml_diff>
--- a/data/profit_data.xlsx
+++ b/data/profit_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O327"/>
+  <dimension ref="A1:O328"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -16190,6 +16190,55 @@
         <v>88281.08</v>
       </c>
     </row>
+    <row r="328">
+      <c r="A328" t="inlineStr">
+        <is>
+          <t>10/18/2026</t>
+        </is>
+      </c>
+      <c r="B328" t="n">
+        <v>14254.16</v>
+      </c>
+      <c r="C328" t="n">
+        <v>0.3482162454400424</v>
+      </c>
+      <c r="D328" t="n">
+        <v>0.6517837545599576</v>
+      </c>
+      <c r="E328" t="n">
+        <v>-195.7</v>
+      </c>
+      <c r="F328" t="n">
+        <v>-8.289999999999999</v>
+      </c>
+      <c r="G328" t="n">
+        <v>-23126.13</v>
+      </c>
+      <c r="H328" t="n">
+        <v>-71.34</v>
+      </c>
+      <c r="I328" t="n">
+        <v>-439.32</v>
+      </c>
+      <c r="J328" t="n">
+        <v>-8.130000000000001</v>
+      </c>
+      <c r="K328" t="n">
+        <v>-23565.45</v>
+      </c>
+      <c r="L328" t="n">
+        <v>-62.31</v>
+      </c>
+      <c r="M328" t="n">
+        <v>0.0376</v>
+      </c>
+      <c r="N328" t="n">
+        <v>0.1202</v>
+      </c>
+      <c r="O328" t="n">
+        <v>88227.64</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update profit files after running on 2026-10-19
</commit_message>
<xml_diff>
--- a/data/profit_data.xlsx
+++ b/data/profit_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O328"/>
+  <dimension ref="A1:O329"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -16239,6 +16239,55 @@
         <v>88227.64</v>
       </c>
     </row>
+    <row r="329">
+      <c r="A329" t="inlineStr">
+        <is>
+          <t>10/19/2026</t>
+        </is>
+      </c>
+      <c r="B329" t="n">
+        <v>14417.8</v>
+      </c>
+      <c r="C329" t="n">
+        <v>0.3470098402120614</v>
+      </c>
+      <c r="D329" t="n">
+        <v>0.6529901597879386</v>
+      </c>
+      <c r="E329" t="n">
+        <v>-166.8</v>
+      </c>
+      <c r="F329" t="n">
+        <v>-7.07</v>
+      </c>
+      <c r="G329" t="n">
+        <v>-23002.08</v>
+      </c>
+      <c r="H329" t="n">
+        <v>-70.95999999999999</v>
+      </c>
+      <c r="I329" t="n">
+        <v>-399.73</v>
+      </c>
+      <c r="J329" t="n">
+        <v>-7.4</v>
+      </c>
+      <c r="K329" t="n">
+        <v>-23401.81</v>
+      </c>
+      <c r="L329" t="n">
+        <v>-61.88</v>
+      </c>
+      <c r="M329" t="n">
+        <v>0.0376</v>
+      </c>
+      <c r="N329" t="n">
+        <v>0.1202</v>
+      </c>
+      <c r="O329" t="n">
+        <v>88227.64</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update profit files after running on 2026-10-20
</commit_message>
<xml_diff>
--- a/data/profit_data.xlsx
+++ b/data/profit_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O329"/>
+  <dimension ref="A1:O330"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -16288,6 +16288,55 @@
         <v>88227.64</v>
       </c>
     </row>
+    <row r="330">
+      <c r="A330" t="inlineStr">
+        <is>
+          <t>10/20/2026</t>
+        </is>
+      </c>
+      <c r="B330" t="n">
+        <v>14979.23</v>
+      </c>
+      <c r="C330" t="n">
+        <v>0.3374569710571964</v>
+      </c>
+      <c r="D330" t="n">
+        <v>0.6625430289428036</v>
+      </c>
+      <c r="E330" t="n">
+        <v>-48.06</v>
+      </c>
+      <c r="F330" t="n">
+        <v>-2.04</v>
+      </c>
+      <c r="G330" t="n">
+        <v>-22492.37</v>
+      </c>
+      <c r="H330" t="n">
+        <v>-69.39</v>
+      </c>
+      <c r="I330" t="n">
+        <v>-348.76</v>
+      </c>
+      <c r="J330" t="n">
+        <v>-6.46</v>
+      </c>
+      <c r="K330" t="n">
+        <v>-22840.37</v>
+      </c>
+      <c r="L330" t="n">
+        <v>-60.39</v>
+      </c>
+      <c r="M330" t="n">
+        <v>0.0376</v>
+      </c>
+      <c r="N330" t="n">
+        <v>0.1202</v>
+      </c>
+      <c r="O330" t="n">
+        <v>88227.64</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update profit files after running on 2026-10-21
</commit_message>
<xml_diff>
--- a/data/profit_data.xlsx
+++ b/data/profit_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O330"/>
+  <dimension ref="A1:O331"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -16337,6 +16337,55 @@
         <v>88227.64</v>
       </c>
     </row>
+    <row r="331">
+      <c r="A331" t="inlineStr">
+        <is>
+          <t>10/21/2026</t>
+        </is>
+      </c>
+      <c r="B331" t="n">
+        <v>15810.66</v>
+      </c>
+      <c r="C331" t="n">
+        <v>0.3274377903100857</v>
+      </c>
+      <c r="D331" t="n">
+        <v>0.6725622096899143</v>
+      </c>
+      <c r="E331" t="n">
+        <v>117.17</v>
+      </c>
+      <c r="F331" t="n">
+        <v>4.96</v>
+      </c>
+      <c r="G331" t="n">
+        <v>-21783.1</v>
+      </c>
+      <c r="H331" t="n">
+        <v>-67.2</v>
+      </c>
+      <c r="I331" t="n">
+        <v>-225.84</v>
+      </c>
+      <c r="J331" t="n">
+        <v>-4.18</v>
+      </c>
+      <c r="K331" t="n">
+        <v>-22008.94</v>
+      </c>
+      <c r="L331" t="n">
+        <v>-58.19</v>
+      </c>
+      <c r="M331" t="n">
+        <v>0.0376</v>
+      </c>
+      <c r="N331" t="n">
+        <v>0.1202</v>
+      </c>
+      <c r="O331" t="n">
+        <v>88227.64</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update profit files after running on 2026-10-22
</commit_message>
<xml_diff>
--- a/data/profit_data.xlsx
+++ b/data/profit_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O331"/>
+  <dimension ref="A1:O332"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -16386,6 +16386,55 @@
         <v>88227.64</v>
       </c>
     </row>
+    <row r="332">
+      <c r="A332" t="inlineStr">
+        <is>
+          <t>10/22/2026</t>
+        </is>
+      </c>
+      <c r="B332" t="n">
+        <v>14894.97</v>
+      </c>
+      <c r="C332" t="n">
+        <v>0.3331657458354852</v>
+      </c>
+      <c r="D332" t="n">
+        <v>0.6668342541645148</v>
+      </c>
+      <c r="E332" t="n">
+        <v>-46.18</v>
+      </c>
+      <c r="F332" t="n">
+        <v>-1.96</v>
+      </c>
+      <c r="G332" t="n">
+        <v>-22484.28</v>
+      </c>
+      <c r="H332" t="n">
+        <v>-69.36</v>
+      </c>
+      <c r="I332" t="n">
+        <v>-440.36</v>
+      </c>
+      <c r="J332" t="n">
+        <v>-8.15</v>
+      </c>
+      <c r="K332" t="n">
+        <v>-22924.64</v>
+      </c>
+      <c r="L332" t="n">
+        <v>-60.62</v>
+      </c>
+      <c r="M332" t="n">
+        <v>0.0376</v>
+      </c>
+      <c r="N332" t="n">
+        <v>0.1202</v>
+      </c>
+      <c r="O332" t="n">
+        <v>88227.64</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update profit files after running on 2026-10-23
</commit_message>
<xml_diff>
--- a/data/profit_data.xlsx
+++ b/data/profit_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O332"/>
+  <dimension ref="A1:O333"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -16435,6 +16435,55 @@
         <v>88227.64</v>
       </c>
     </row>
+    <row r="333">
+      <c r="A333" t="inlineStr">
+        <is>
+          <t>10/23/2026</t>
+        </is>
+      </c>
+      <c r="B333" t="n">
+        <v>14999.91</v>
+      </c>
+      <c r="C333" t="n">
+        <v>0.3333033133744998</v>
+      </c>
+      <c r="D333" t="n">
+        <v>0.6666966866255002</v>
+      </c>
+      <c r="E333" t="n">
+        <v>-42.75</v>
+      </c>
+      <c r="F333" t="n">
+        <v>-1.77</v>
+      </c>
+      <c r="G333" t="n">
+        <v>-22466.37</v>
+      </c>
+      <c r="H333" t="n">
+        <v>-69.2</v>
+      </c>
+      <c r="I333" t="n">
+        <v>-403.5</v>
+      </c>
+      <c r="J333" t="n">
+        <v>-7.47</v>
+      </c>
+      <c r="K333" t="n">
+        <v>-22869.7</v>
+      </c>
+      <c r="L333" t="n">
+        <v>-60.39</v>
+      </c>
+      <c r="M333" t="n">
+        <v>0.0376</v>
+      </c>
+      <c r="N333" t="n">
+        <v>0.1198</v>
+      </c>
+      <c r="O333" t="n">
+        <v>88227.64</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update profit files after running on 2026-10-24
</commit_message>
<xml_diff>
--- a/data/profit_data.xlsx
+++ b/data/profit_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O333"/>
+  <dimension ref="A1:O334"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -16484,6 +16484,55 @@
         <v>88227.64</v>
       </c>
     </row>
+    <row r="334">
+      <c r="A334" t="inlineStr">
+        <is>
+          <t>10/24/2026</t>
+        </is>
+      </c>
+      <c r="B334" t="n">
+        <v>14455.4</v>
+      </c>
+      <c r="C334" t="n">
+        <v>0.336499833483222</v>
+      </c>
+      <c r="D334" t="n">
+        <v>0.663500166516778</v>
+      </c>
+      <c r="E334" t="n">
+        <v>-139.62</v>
+      </c>
+      <c r="F334" t="n">
+        <v>-5.79</v>
+      </c>
+      <c r="G334" t="n">
+        <v>-22875.6</v>
+      </c>
+      <c r="H334" t="n">
+        <v>-70.45999999999999</v>
+      </c>
+      <c r="I334" t="n">
+        <v>-538.61</v>
+      </c>
+      <c r="J334" t="n">
+        <v>-9.970000000000001</v>
+      </c>
+      <c r="K334" t="n">
+        <v>-23414.21</v>
+      </c>
+      <c r="L334" t="n">
+        <v>-61.83</v>
+      </c>
+      <c r="M334" t="n">
+        <v>0.0376</v>
+      </c>
+      <c r="N334" t="n">
+        <v>0.1198</v>
+      </c>
+      <c r="O334" t="n">
+        <v>88227.64</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update profit files after running on 2026-10-25
</commit_message>
<xml_diff>
--- a/data/profit_data.xlsx
+++ b/data/profit_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O334"/>
+  <dimension ref="A1:O335"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -16533,6 +16533,55 @@
         <v>88227.64</v>
       </c>
     </row>
+    <row r="335">
+      <c r="A335" t="inlineStr">
+        <is>
+          <t>10/25/2026</t>
+        </is>
+      </c>
+      <c r="B335" t="n">
+        <v>14723.25</v>
+      </c>
+      <c r="C335" t="n">
+        <v>0.338446513467733</v>
+      </c>
+      <c r="D335" t="n">
+        <v>0.661553486532267</v>
+      </c>
+      <c r="E335" t="n">
+        <v>-104.33</v>
+      </c>
+      <c r="F335" t="n">
+        <v>-4.33</v>
+      </c>
+      <c r="G335" t="n">
+        <v>-22726.54</v>
+      </c>
+      <c r="H335" t="n">
+        <v>-70</v>
+      </c>
+      <c r="I335" t="n">
+        <v>-469.82</v>
+      </c>
+      <c r="J335" t="n">
+        <v>-8.619999999999999</v>
+      </c>
+      <c r="K335" t="n">
+        <v>-23196.36</v>
+      </c>
+      <c r="L335" t="n">
+        <v>-61.17</v>
+      </c>
+      <c r="M335" t="n">
+        <v>0.0376</v>
+      </c>
+      <c r="N335" t="n">
+        <v>0.1198</v>
+      </c>
+      <c r="O335" t="n">
+        <v>88163.49000000001</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update profit files after running on 2026-10-26
</commit_message>
<xml_diff>
--- a/data/profit_data.xlsx
+++ b/data/profit_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O335"/>
+  <dimension ref="A1:O336"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -16582,6 +16582,55 @@
         <v>88163.49000000001</v>
       </c>
     </row>
+    <row r="336">
+      <c r="A336" t="inlineStr">
+        <is>
+          <t>10/26/2026</t>
+        </is>
+      </c>
+      <c r="B336" t="n">
+        <v>14545.71</v>
+      </c>
+      <c r="C336" t="n">
+        <v>0.3406193749957029</v>
+      </c>
+      <c r="D336" t="n">
+        <v>0.6593806250042971</v>
+      </c>
+      <c r="E336" t="n">
+        <v>-139.62</v>
+      </c>
+      <c r="F336" t="n">
+        <v>-5.79</v>
+      </c>
+      <c r="G336" t="n">
+        <v>-22875.6</v>
+      </c>
+      <c r="H336" t="n">
+        <v>-70.45999999999999</v>
+      </c>
+      <c r="I336" t="n">
+        <v>-498.3</v>
+      </c>
+      <c r="J336" t="n">
+        <v>-9.140000000000001</v>
+      </c>
+      <c r="K336" t="n">
+        <v>-23373.9</v>
+      </c>
+      <c r="L336" t="n">
+        <v>-61.64</v>
+      </c>
+      <c r="M336" t="n">
+        <v>0.0376</v>
+      </c>
+      <c r="N336" t="n">
+        <v>0.1198</v>
+      </c>
+      <c r="O336" t="n">
+        <v>88163.49000000001</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update profit files after running on 2026-10-27
</commit_message>
<xml_diff>
--- a/data/profit_data.xlsx
+++ b/data/profit_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O336"/>
+  <dimension ref="A1:O337"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -16631,6 +16631,55 @@
         <v>88163.49000000001</v>
       </c>
     </row>
+    <row r="337">
+      <c r="A337" t="inlineStr">
+        <is>
+          <t>10/27/2026</t>
+        </is>
+      </c>
+      <c r="B337" t="n">
+        <v>14537.08</v>
+      </c>
+      <c r="C337" t="n">
+        <v>0.3428378699118526</v>
+      </c>
+      <c r="D337" t="n">
+        <v>0.6571621300881474</v>
+      </c>
+      <c r="E337" t="n">
+        <v>-148.6</v>
+      </c>
+      <c r="F337" t="n">
+        <v>-6.17</v>
+      </c>
+      <c r="G337" t="n">
+        <v>-22913.54</v>
+      </c>
+      <c r="H337" t="n">
+        <v>-70.58</v>
+      </c>
+      <c r="I337" t="n">
+        <v>-468.99</v>
+      </c>
+      <c r="J337" t="n">
+        <v>-8.6</v>
+      </c>
+      <c r="K337" t="n">
+        <v>-23382.53</v>
+      </c>
+      <c r="L337" t="n">
+        <v>-61.66</v>
+      </c>
+      <c r="M337" t="n">
+        <v>0.0376</v>
+      </c>
+      <c r="N337" t="n">
+        <v>0.1198</v>
+      </c>
+      <c r="O337" t="n">
+        <v>88163.49000000001</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update profit files after running on 2026-10-28
</commit_message>
<xml_diff>
--- a/data/profit_data.xlsx
+++ b/data/profit_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O337"/>
+  <dimension ref="A1:O338"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -16680,6 +16680,55 @@
         <v>88163.49000000001</v>
       </c>
     </row>
+    <row r="338">
+      <c r="A338" t="inlineStr">
+        <is>
+          <t>10/28/2026</t>
+        </is>
+      </c>
+      <c r="B338" t="n">
+        <v>14678.33</v>
+      </c>
+      <c r="C338" t="n">
+        <v>0.3409931976152395</v>
+      </c>
+      <c r="D338" t="n">
+        <v>0.6590068023847605</v>
+      </c>
+      <c r="E338" t="n">
+        <v>-120.37</v>
+      </c>
+      <c r="F338" t="n">
+        <v>-4.99</v>
+      </c>
+      <c r="G338" t="n">
+        <v>-22794.3</v>
+      </c>
+      <c r="H338" t="n">
+        <v>-70.20999999999999</v>
+      </c>
+      <c r="I338" t="n">
+        <v>-447.98</v>
+      </c>
+      <c r="J338" t="n">
+        <v>-8.220000000000001</v>
+      </c>
+      <c r="K338" t="n">
+        <v>-23242.28</v>
+      </c>
+      <c r="L338" t="n">
+        <v>-61.29</v>
+      </c>
+      <c r="M338" t="n">
+        <v>0.0376</v>
+      </c>
+      <c r="N338" t="n">
+        <v>0.1198</v>
+      </c>
+      <c r="O338" t="n">
+        <v>88163.49000000001</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update profit files after running on 2026-10-29
</commit_message>
<xml_diff>
--- a/data/profit_data.xlsx
+++ b/data/profit_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O338"/>
+  <dimension ref="A1:O339"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -16729,6 +16729,55 @@
         <v>88163.49000000001</v>
       </c>
     </row>
+    <row r="339">
+      <c r="A339" t="inlineStr">
+        <is>
+          <t>10/29/2026</t>
+        </is>
+      </c>
+      <c r="B339" t="n">
+        <v>14805.31</v>
+      </c>
+      <c r="C339" t="n">
+        <v>0.3373541930165024</v>
+      </c>
+      <c r="D339" t="n">
+        <v>0.6626458069834976</v>
+      </c>
+      <c r="E339" t="n">
+        <v>-87.65000000000001</v>
+      </c>
+      <c r="F339" t="n">
+        <v>-3.64</v>
+      </c>
+      <c r="G339" t="n">
+        <v>-22656.08</v>
+      </c>
+      <c r="H339" t="n">
+        <v>-69.78</v>
+      </c>
+      <c r="I339" t="n">
+        <v>-458.21</v>
+      </c>
+      <c r="J339" t="n">
+        <v>-8.4</v>
+      </c>
+      <c r="K339" t="n">
+        <v>-23114.29</v>
+      </c>
+      <c r="L339" t="n">
+        <v>-60.96</v>
+      </c>
+      <c r="M339" t="n">
+        <v>0.0376</v>
+      </c>
+      <c r="N339" t="n">
+        <v>0.1198</v>
+      </c>
+      <c r="O339" t="n">
+        <v>88163.49000000001</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update profit files after running on 2026-10-30
</commit_message>
<xml_diff>
--- a/data/profit_data.xlsx
+++ b/data/profit_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O339"/>
+  <dimension ref="A1:O340"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -16778,6 +16778,55 @@
         <v>88163.49000000001</v>
       </c>
     </row>
+    <row r="340">
+      <c r="A340" t="inlineStr">
+        <is>
+          <t>10/30/2026</t>
+        </is>
+      </c>
+      <c r="B340" t="n">
+        <v>13722.1</v>
+      </c>
+      <c r="C340" t="n">
+        <v>0.3478265279737371</v>
+      </c>
+      <c r="D340" t="n">
+        <v>0.6521734720262629</v>
+      </c>
+      <c r="E340" t="n">
+        <v>-306.16</v>
+      </c>
+      <c r="F340" t="n">
+        <v>-12.45</v>
+      </c>
+      <c r="G340" t="n">
+        <v>-23567.57</v>
+      </c>
+      <c r="H340" t="n">
+        <v>-72.48</v>
+      </c>
+      <c r="I340" t="n">
+        <v>-679.9400000000001</v>
+      </c>
+      <c r="J340" t="n">
+        <v>-12.47</v>
+      </c>
+      <c r="K340" t="n">
+        <v>-24247.51</v>
+      </c>
+      <c r="L340" t="n">
+        <v>-63.86</v>
+      </c>
+      <c r="M340" t="n">
+        <v>0.0375</v>
+      </c>
+      <c r="N340" t="n">
+        <v>0.1194</v>
+      </c>
+      <c r="O340" t="n">
+        <v>88163.49000000001</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update profit files after running on 2026-10-31
</commit_message>
<xml_diff>
--- a/data/profit_data.xlsx
+++ b/data/profit_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O340"/>
+  <dimension ref="A1:O341"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -16827,6 +16827,55 @@
         <v>88163.49000000001</v>
       </c>
     </row>
+    <row r="341">
+      <c r="A341" t="inlineStr">
+        <is>
+          <t>10/31/2026</t>
+        </is>
+      </c>
+      <c r="B341" t="n">
+        <v>13782.44</v>
+      </c>
+      <c r="C341" t="n">
+        <v>0.3477168531816199</v>
+      </c>
+      <c r="D341" t="n">
+        <v>0.6522831468183801</v>
+      </c>
+      <c r="E341" t="n">
+        <v>-296.33</v>
+      </c>
+      <c r="F341" t="n">
+        <v>-12.05</v>
+      </c>
+      <c r="G341" t="n">
+        <v>-23526.7</v>
+      </c>
+      <c r="H341" t="n">
+        <v>-72.34999999999999</v>
+      </c>
+      <c r="I341" t="n">
+        <v>-660.46</v>
+      </c>
+      <c r="J341" t="n">
+        <v>-12.11</v>
+      </c>
+      <c r="K341" t="n">
+        <v>-24187.16</v>
+      </c>
+      <c r="L341" t="n">
+        <v>-63.7</v>
+      </c>
+      <c r="M341" t="n">
+        <v>0.0375</v>
+      </c>
+      <c r="N341" t="n">
+        <v>0.1194</v>
+      </c>
+      <c r="O341" t="n">
+        <v>88163.49000000001</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>